<commit_message>
Added English from the 'AllRight2' method. Added the ability to learn both directions.
</commit_message>
<xml_diff>
--- a/python_scripts/words.xlsx
+++ b/python_scripts/words.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3082" uniqueCount="1893">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3454" uniqueCount="2171">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -5699,6 +5699,840 @@
   </si>
   <si>
     <t xml:space="preserve">ergo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">amount of</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hoeveelheid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">carbohydrates</t>
+  </si>
+  <si>
+    <t xml:space="preserve">koolhydraten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cauliflower</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bloemkool</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">to contain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bevatten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cottage cheese</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kwark</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">deposit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">statiegeld/borg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">food label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">voedingsetiket</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">listed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">opgesomd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nutrition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">voeding</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_010</t>
+  </si>
+  <si>
+    <t xml:space="preserve">packaged</t>
+  </si>
+  <si>
+    <t xml:space="preserve">verpakt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">popsicle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ijslolly</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_012</t>
+  </si>
+  <si>
+    <t xml:space="preserve">produce (section)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(afdeling) groenten en fruit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_013</t>
+  </si>
+  <si>
+    <t xml:space="preserve">saturated fat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">verzadigd vet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_014</t>
+  </si>
+  <si>
+    <t xml:space="preserve">serving</t>
+  </si>
+  <si>
+    <t xml:space="preserve">portie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_015</t>
+  </si>
+  <si>
+    <t xml:space="preserve">shelf stacker</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vakkenvuller</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_016</t>
+  </si>
+  <si>
+    <t xml:space="preserve">skimmed milk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">magere melk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_017</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dairy (section)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(afdeling) melkproducten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_018</t>
+  </si>
+  <si>
+    <t xml:space="preserve">supplies</t>
+  </si>
+  <si>
+    <t xml:space="preserve">benodigdheden</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_019</t>
+  </si>
+  <si>
+    <t xml:space="preserve">aisle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gang(pad)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">checkout/cash register</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kassa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_021</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cashier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kassamedewerker</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_022</t>
+  </si>
+  <si>
+    <t xml:space="preserve">customer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">klant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">discount</t>
+  </si>
+  <si>
+    <t xml:space="preserve">korting</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">to borrow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lenen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">solution</t>
+  </si>
+  <si>
+    <t xml:space="preserve">oplossing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">shelf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">schap/plank</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">butcher’s shop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">slagerij</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_028</t>
+  </si>
+  <si>
+    <t xml:space="preserve">counter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">toonbank</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_029</t>
+  </si>
+  <si>
+    <t xml:space="preserve">packaging</t>
+  </si>
+  <si>
+    <t xml:space="preserve">verpakking</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_030</t>
+  </si>
+  <si>
+    <t xml:space="preserve">to waste</t>
+  </si>
+  <si>
+    <t xml:space="preserve">verspillen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_031</t>
+  </si>
+  <si>
+    <t xml:space="preserve">to weigh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wegen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_032</t>
+  </si>
+  <si>
+    <t xml:space="preserve">shopping cart</t>
+  </si>
+  <si>
+    <t xml:space="preserve">winkelkarretje</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_033</t>
+  </si>
+  <si>
+    <t xml:space="preserve">shopping basket</t>
+  </si>
+  <si>
+    <t xml:space="preserve">winkelmandje</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_034</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(bi-)annual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(twee-)jaarlijks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_035</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bold</t>
+  </si>
+  <si>
+    <t xml:space="preserve">opvallend</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_036</t>
+  </si>
+  <si>
+    <t xml:space="preserve">casual (clothes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">informeel/vrijetijds-(kleding)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_037</t>
+  </si>
+  <si>
+    <t xml:space="preserve">to display</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tonen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_038</t>
+  </si>
+  <si>
+    <t xml:space="preserve">edgy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gewaagd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_039</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fabric</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stof/materiaal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_040</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fibre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vezel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_041</t>
+  </si>
+  <si>
+    <t xml:space="preserve">garment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kledingstuk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_042</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gown</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lange jurk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_043</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hem</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zoom</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_044</t>
+  </si>
+  <si>
+    <t xml:space="preserve">high street</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(winkels) voor het grote publiek</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_045</t>
+  </si>
+  <si>
+    <t xml:space="preserve">old-fashioned</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ouderwets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_046</t>
+  </si>
+  <si>
+    <t xml:space="preserve">retailer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">detailhandelaar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_047</t>
+  </si>
+  <si>
+    <t xml:space="preserve">seam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">naad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_048</t>
+  </si>
+  <si>
+    <t xml:space="preserve">to showcase</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tentoonstellen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_049</t>
+  </si>
+  <si>
+    <t xml:space="preserve">to sift through</t>
+  </si>
+  <si>
+    <t xml:space="preserve">doorzoeken</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_050</t>
+  </si>
+  <si>
+    <t xml:space="preserve">thrift shop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kringloopwinkel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_051</t>
+  </si>
+  <si>
+    <t xml:space="preserve">catwalk/runway</t>
+  </si>
+  <si>
+    <t xml:space="preserve">catwalk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_052</t>
+  </si>
+  <si>
+    <t xml:space="preserve">classy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">chic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_053</t>
+  </si>
+  <si>
+    <t xml:space="preserve">to draw attention</t>
+  </si>
+  <si>
+    <t xml:space="preserve">de aandacht trekken</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_054</t>
+  </si>
+  <si>
+    <t xml:space="preserve">knit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gebreid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_055</t>
+  </si>
+  <si>
+    <t xml:space="preserve">to be inspired by</t>
+  </si>
+  <si>
+    <t xml:space="preserve">geïnspireerd worden door</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_056</t>
+  </si>
+  <si>
+    <t xml:space="preserve">good cause</t>
+  </si>
+  <si>
+    <t xml:space="preserve">goed doel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_057</t>
+  </si>
+  <si>
+    <t xml:space="preserve">well-dressed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">goed gekleed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_058</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cotton</t>
+  </si>
+  <si>
+    <t xml:space="preserve">katoen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_059</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bargain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">koopje</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_060</t>
+  </si>
+  <si>
+    <t xml:space="preserve">leather</t>
+  </si>
+  <si>
+    <t xml:space="preserve">leer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_061</t>
+  </si>
+  <si>
+    <t xml:space="preserve">linen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">linnen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_062</t>
+  </si>
+  <si>
+    <t xml:space="preserve">label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">merk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_063</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pattern</t>
+  </si>
+  <si>
+    <t xml:space="preserve">patroon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_064</t>
+  </si>
+  <si>
+    <t xml:space="preserve">denim</t>
+  </si>
+  <si>
+    <t xml:space="preserve">spijkerstof</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_065</t>
+  </si>
+  <si>
+    <t xml:space="preserve">style</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stijl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_066</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wool</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wol</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_067</t>
+  </si>
+  <si>
+    <t xml:space="preserve">silk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zijde</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_068</t>
+  </si>
+  <si>
+    <t xml:space="preserve">accessories</t>
+  </si>
+  <si>
+    <t xml:space="preserve">accessoires</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_069</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bank holiday</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nationale feestdag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_070</t>
+  </si>
+  <si>
+    <t xml:space="preserve">christening</t>
+  </si>
+  <si>
+    <t xml:space="preserve">doop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_071</t>
+  </si>
+  <si>
+    <t xml:space="preserve">festivity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">feestelijkheid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_072</t>
+  </si>
+  <si>
+    <t xml:space="preserve">to honour</t>
+  </si>
+  <si>
+    <t xml:space="preserve">eren</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_073</t>
+  </si>
+  <si>
+    <t xml:space="preserve">leprechaun</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(Ierse) elf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_074</t>
+  </si>
+  <si>
+    <t xml:space="preserve">to originate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ontstaan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_075</t>
+  </si>
+  <si>
+    <t xml:space="preserve">patron saint</t>
+  </si>
+  <si>
+    <t xml:space="preserve">beschermheilige</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_076</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pentecost</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pinksteren</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_077</t>
+  </si>
+  <si>
+    <t xml:space="preserve">to recognise</t>
+  </si>
+  <si>
+    <t xml:space="preserve">erkennen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_078</t>
+  </si>
+  <si>
+    <t xml:space="preserve">touching</t>
+  </si>
+  <si>
+    <t xml:space="preserve">aandoenlijk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_079</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gift; present</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cadeautje</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_080</t>
+  </si>
+  <si>
+    <t xml:space="preserve">graduation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">diploma-uitreiking</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_081</t>
+  </si>
+  <si>
+    <t xml:space="preserve">to dress up</t>
+  </si>
+  <si>
+    <t xml:space="preserve">formeel kleden/verkleden</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_082</t>
+  </si>
+  <si>
+    <t xml:space="preserve">custom</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gewoonte/gebruik</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_083</t>
+  </si>
+  <si>
+    <t xml:space="preserve">to wrap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">inpakken</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_084</t>
+  </si>
+  <si>
+    <t xml:space="preserve">anniversary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jubileum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_085</t>
+  </si>
+  <si>
+    <t xml:space="preserve">public holiday</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_086</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Easter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pasen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_087</t>
+  </si>
+  <si>
+    <t xml:space="preserve">to take place</t>
+  </si>
+  <si>
+    <t xml:space="preserve">plaatsvinden</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_088</t>
+  </si>
+  <si>
+    <t xml:space="preserve">to invite</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_089</t>
+  </si>
+  <si>
+    <t xml:space="preserve">invitation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">uitnodiging</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_090</t>
+  </si>
+  <si>
+    <t xml:space="preserve">to gather</t>
+  </si>
+  <si>
+    <t xml:space="preserve">verzamelen/samenkomen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_091</t>
+  </si>
+  <si>
+    <t xml:space="preserve">to celebrate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vieren</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_092</t>
+  </si>
+  <si>
+    <t xml:space="preserve">day off</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vrije dag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllRight2_093</t>
+  </si>
+  <si>
+    <t xml:space="preserve">to be embarrassed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zich generen (schamen)</t>
   </si>
 </sst>
 </file>
@@ -5975,7 +6809,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F580"/>
+  <dimension ref="A1:F673"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16.05"/>
@@ -16391,6 +17225,1587 @@
         <v>240</v>
       </c>
     </row>
+    <row r="581" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A581" s="1" t="s">
+        <v>1893</v>
+      </c>
+      <c r="B581" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C581" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D581" s="0" t="s">
+        <v>1895</v>
+      </c>
+      <c r="E581" s="0" t="s">
+        <v>1896</v>
+      </c>
+    </row>
+    <row r="582" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A582" s="1" t="s">
+        <v>1897</v>
+      </c>
+      <c r="B582" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C582" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D582" s="0" t="s">
+        <v>1898</v>
+      </c>
+      <c r="E582" s="0" t="s">
+        <v>1899</v>
+      </c>
+    </row>
+    <row r="583" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A583" s="1" t="s">
+        <v>1900</v>
+      </c>
+      <c r="B583" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C583" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D583" s="0" t="s">
+        <v>1901</v>
+      </c>
+      <c r="E583" s="0" t="s">
+        <v>1902</v>
+      </c>
+    </row>
+    <row r="584" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A584" s="1" t="s">
+        <v>1903</v>
+      </c>
+      <c r="B584" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C584" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D584" s="0" t="s">
+        <v>1904</v>
+      </c>
+      <c r="E584" s="0" t="s">
+        <v>1905</v>
+      </c>
+    </row>
+    <row r="585" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A585" s="1" t="s">
+        <v>1906</v>
+      </c>
+      <c r="B585" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C585" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D585" s="0" t="s">
+        <v>1907</v>
+      </c>
+      <c r="E585" s="0" t="s">
+        <v>1908</v>
+      </c>
+    </row>
+    <row r="586" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A586" s="1" t="s">
+        <v>1909</v>
+      </c>
+      <c r="B586" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C586" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D586" s="0" t="s">
+        <v>1910</v>
+      </c>
+      <c r="E586" s="0" t="s">
+        <v>1911</v>
+      </c>
+    </row>
+    <row r="587" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A587" s="1" t="s">
+        <v>1912</v>
+      </c>
+      <c r="B587" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C587" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D587" s="0" t="s">
+        <v>1913</v>
+      </c>
+      <c r="E587" s="0" t="s">
+        <v>1914</v>
+      </c>
+    </row>
+    <row r="588" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A588" s="1" t="s">
+        <v>1915</v>
+      </c>
+      <c r="B588" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C588" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D588" s="0" t="s">
+        <v>1916</v>
+      </c>
+      <c r="E588" s="0" t="s">
+        <v>1917</v>
+      </c>
+    </row>
+    <row r="589" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A589" s="1" t="s">
+        <v>1918</v>
+      </c>
+      <c r="B589" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C589" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D589" s="0" t="s">
+        <v>1919</v>
+      </c>
+      <c r="E589" s="0" t="s">
+        <v>1920</v>
+      </c>
+    </row>
+    <row r="590" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A590" s="1" t="s">
+        <v>1921</v>
+      </c>
+      <c r="B590" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C590" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D590" s="0" t="s">
+        <v>1922</v>
+      </c>
+      <c r="E590" s="0" t="s">
+        <v>1923</v>
+      </c>
+    </row>
+    <row r="591" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A591" s="1" t="s">
+        <v>1924</v>
+      </c>
+      <c r="B591" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C591" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D591" s="0" t="s">
+        <v>1925</v>
+      </c>
+      <c r="E591" s="0" t="s">
+        <v>1926</v>
+      </c>
+    </row>
+    <row r="592" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A592" s="1" t="s">
+        <v>1927</v>
+      </c>
+      <c r="B592" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C592" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D592" s="0" t="s">
+        <v>1928</v>
+      </c>
+      <c r="E592" s="0" t="s">
+        <v>1929</v>
+      </c>
+    </row>
+    <row r="593" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A593" s="1" t="s">
+        <v>1930</v>
+      </c>
+      <c r="B593" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C593" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D593" s="0" t="s">
+        <v>1931</v>
+      </c>
+      <c r="E593" s="0" t="s">
+        <v>1932</v>
+      </c>
+    </row>
+    <row r="594" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A594" s="1" t="s">
+        <v>1933</v>
+      </c>
+      <c r="B594" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C594" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D594" s="0" t="s">
+        <v>1934</v>
+      </c>
+      <c r="E594" s="0" t="s">
+        <v>1935</v>
+      </c>
+    </row>
+    <row r="595" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A595" s="1" t="s">
+        <v>1936</v>
+      </c>
+      <c r="B595" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C595" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D595" s="0" t="s">
+        <v>1937</v>
+      </c>
+      <c r="E595" s="0" t="s">
+        <v>1938</v>
+      </c>
+    </row>
+    <row r="596" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A596" s="1" t="s">
+        <v>1939</v>
+      </c>
+      <c r="B596" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C596" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D596" s="0" t="s">
+        <v>1940</v>
+      </c>
+      <c r="E596" s="0" t="s">
+        <v>1941</v>
+      </c>
+    </row>
+    <row r="597" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A597" s="1" t="s">
+        <v>1942</v>
+      </c>
+      <c r="B597" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C597" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D597" s="0" t="s">
+        <v>1943</v>
+      </c>
+      <c r="E597" s="0" t="s">
+        <v>1944</v>
+      </c>
+    </row>
+    <row r="598" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A598" s="1" t="s">
+        <v>1945</v>
+      </c>
+      <c r="B598" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C598" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D598" s="0" t="s">
+        <v>1946</v>
+      </c>
+      <c r="E598" s="0" t="s">
+        <v>1947</v>
+      </c>
+    </row>
+    <row r="599" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A599" s="1" t="s">
+        <v>1948</v>
+      </c>
+      <c r="B599" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C599" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D599" s="0" t="s">
+        <v>1949</v>
+      </c>
+      <c r="E599" s="0" t="s">
+        <v>1950</v>
+      </c>
+    </row>
+    <row r="600" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A600" s="1" t="s">
+        <v>1951</v>
+      </c>
+      <c r="B600" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C600" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D600" s="0" t="s">
+        <v>1952</v>
+      </c>
+      <c r="E600" s="0" t="s">
+        <v>1953</v>
+      </c>
+    </row>
+    <row r="601" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A601" s="1" t="s">
+        <v>1954</v>
+      </c>
+      <c r="B601" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C601" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D601" s="0" t="s">
+        <v>1955</v>
+      </c>
+      <c r="E601" s="0" t="s">
+        <v>1956</v>
+      </c>
+    </row>
+    <row r="602" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A602" s="1" t="s">
+        <v>1957</v>
+      </c>
+      <c r="B602" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C602" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D602" s="0" t="s">
+        <v>1958</v>
+      </c>
+      <c r="E602" s="0" t="s">
+        <v>1959</v>
+      </c>
+    </row>
+    <row r="603" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A603" s="1" t="s">
+        <v>1960</v>
+      </c>
+      <c r="B603" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C603" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D603" s="0" t="s">
+        <v>1961</v>
+      </c>
+      <c r="E603" s="0" t="s">
+        <v>1962</v>
+      </c>
+    </row>
+    <row r="604" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A604" s="1" t="s">
+        <v>1963</v>
+      </c>
+      <c r="B604" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C604" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D604" s="0" t="s">
+        <v>1964</v>
+      </c>
+      <c r="E604" s="0" t="s">
+        <v>1965</v>
+      </c>
+    </row>
+    <row r="605" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A605" s="1" t="s">
+        <v>1966</v>
+      </c>
+      <c r="B605" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C605" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D605" s="0" t="s">
+        <v>1967</v>
+      </c>
+      <c r="E605" s="0" t="s">
+        <v>1968</v>
+      </c>
+    </row>
+    <row r="606" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A606" s="1" t="s">
+        <v>1969</v>
+      </c>
+      <c r="B606" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C606" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D606" s="0" t="s">
+        <v>1970</v>
+      </c>
+      <c r="E606" s="0" t="s">
+        <v>1971</v>
+      </c>
+    </row>
+    <row r="607" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A607" s="1" t="s">
+        <v>1972</v>
+      </c>
+      <c r="B607" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C607" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D607" s="0" t="s">
+        <v>1973</v>
+      </c>
+      <c r="E607" s="0" t="s">
+        <v>1974</v>
+      </c>
+    </row>
+    <row r="608" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A608" s="1" t="s">
+        <v>1975</v>
+      </c>
+      <c r="B608" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C608" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D608" s="0" t="s">
+        <v>1976</v>
+      </c>
+      <c r="E608" s="0" t="s">
+        <v>1977</v>
+      </c>
+    </row>
+    <row r="609" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A609" s="1" t="s">
+        <v>1978</v>
+      </c>
+      <c r="B609" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C609" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D609" s="0" t="s">
+        <v>1979</v>
+      </c>
+      <c r="E609" s="0" t="s">
+        <v>1980</v>
+      </c>
+    </row>
+    <row r="610" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A610" s="1" t="s">
+        <v>1981</v>
+      </c>
+      <c r="B610" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C610" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D610" s="0" t="s">
+        <v>1982</v>
+      </c>
+      <c r="E610" s="0" t="s">
+        <v>1983</v>
+      </c>
+    </row>
+    <row r="611" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A611" s="1" t="s">
+        <v>1984</v>
+      </c>
+      <c r="B611" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C611" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D611" s="0" t="s">
+        <v>1985</v>
+      </c>
+      <c r="E611" s="0" t="s">
+        <v>1986</v>
+      </c>
+    </row>
+    <row r="612" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A612" s="1" t="s">
+        <v>1987</v>
+      </c>
+      <c r="B612" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C612" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D612" s="0" t="s">
+        <v>1988</v>
+      </c>
+      <c r="E612" s="0" t="s">
+        <v>1989</v>
+      </c>
+    </row>
+    <row r="613" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A613" s="1" t="s">
+        <v>1990</v>
+      </c>
+      <c r="B613" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C613" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D613" s="0" t="s">
+        <v>1991</v>
+      </c>
+      <c r="E613" s="0" t="s">
+        <v>1992</v>
+      </c>
+    </row>
+    <row r="614" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A614" s="1" t="s">
+        <v>1993</v>
+      </c>
+      <c r="B614" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C614" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D614" s="0" t="s">
+        <v>1994</v>
+      </c>
+      <c r="E614" s="0" t="s">
+        <v>1995</v>
+      </c>
+    </row>
+    <row r="615" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A615" s="1" t="s">
+        <v>1996</v>
+      </c>
+      <c r="B615" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C615" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D615" s="0" t="s">
+        <v>1997</v>
+      </c>
+      <c r="E615" s="0" t="s">
+        <v>1998</v>
+      </c>
+    </row>
+    <row r="616" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A616" s="1" t="s">
+        <v>1999</v>
+      </c>
+      <c r="B616" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C616" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D616" s="0" t="s">
+        <v>2000</v>
+      </c>
+      <c r="E616" s="0" t="s">
+        <v>2001</v>
+      </c>
+    </row>
+    <row r="617" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A617" s="1" t="s">
+        <v>2002</v>
+      </c>
+      <c r="B617" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C617" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D617" s="0" t="s">
+        <v>2003</v>
+      </c>
+      <c r="E617" s="0" t="s">
+        <v>2004</v>
+      </c>
+    </row>
+    <row r="618" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A618" s="1" t="s">
+        <v>2005</v>
+      </c>
+      <c r="B618" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C618" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D618" s="0" t="s">
+        <v>2006</v>
+      </c>
+      <c r="E618" s="0" t="s">
+        <v>2007</v>
+      </c>
+    </row>
+    <row r="619" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A619" s="1" t="s">
+        <v>2008</v>
+      </c>
+      <c r="B619" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C619" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D619" s="0" t="s">
+        <v>2009</v>
+      </c>
+      <c r="E619" s="0" t="s">
+        <v>2010</v>
+      </c>
+    </row>
+    <row r="620" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A620" s="1" t="s">
+        <v>2011</v>
+      </c>
+      <c r="B620" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C620" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D620" s="0" t="s">
+        <v>2012</v>
+      </c>
+      <c r="E620" s="0" t="s">
+        <v>2013</v>
+      </c>
+    </row>
+    <row r="621" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A621" s="1" t="s">
+        <v>2014</v>
+      </c>
+      <c r="B621" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C621" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D621" s="0" t="s">
+        <v>2015</v>
+      </c>
+      <c r="E621" s="0" t="s">
+        <v>2016</v>
+      </c>
+    </row>
+    <row r="622" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A622" s="1" t="s">
+        <v>2017</v>
+      </c>
+      <c r="B622" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C622" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D622" s="0" t="s">
+        <v>2018</v>
+      </c>
+      <c r="E622" s="0" t="s">
+        <v>2019</v>
+      </c>
+    </row>
+    <row r="623" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A623" s="1" t="s">
+        <v>2020</v>
+      </c>
+      <c r="B623" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C623" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D623" s="0" t="s">
+        <v>2021</v>
+      </c>
+      <c r="E623" s="0" t="s">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="624" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A624" s="1" t="s">
+        <v>2023</v>
+      </c>
+      <c r="B624" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C624" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D624" s="0" t="s">
+        <v>2024</v>
+      </c>
+      <c r="E624" s="0" t="s">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="625" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A625" s="1" t="s">
+        <v>2026</v>
+      </c>
+      <c r="B625" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C625" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D625" s="0" t="s">
+        <v>2027</v>
+      </c>
+      <c r="E625" s="0" t="s">
+        <v>2028</v>
+      </c>
+    </row>
+    <row r="626" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A626" s="1" t="s">
+        <v>2029</v>
+      </c>
+      <c r="B626" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C626" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D626" s="0" t="s">
+        <v>2030</v>
+      </c>
+      <c r="E626" s="0" t="s">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="627" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A627" s="1" t="s">
+        <v>2032</v>
+      </c>
+      <c r="B627" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C627" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D627" s="0" t="s">
+        <v>2033</v>
+      </c>
+      <c r="E627" s="0" t="s">
+        <v>2034</v>
+      </c>
+    </row>
+    <row r="628" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A628" s="1" t="s">
+        <v>2035</v>
+      </c>
+      <c r="B628" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C628" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D628" s="0" t="s">
+        <v>2036</v>
+      </c>
+      <c r="E628" s="0" t="s">
+        <v>2037</v>
+      </c>
+    </row>
+    <row r="629" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A629" s="1" t="s">
+        <v>2038</v>
+      </c>
+      <c r="B629" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C629" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D629" s="0" t="s">
+        <v>2039</v>
+      </c>
+      <c r="E629" s="0" t="s">
+        <v>2040</v>
+      </c>
+    </row>
+    <row r="630" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A630" s="1" t="s">
+        <v>2041</v>
+      </c>
+      <c r="B630" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C630" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D630" s="0" t="s">
+        <v>2042</v>
+      </c>
+      <c r="E630" s="0" t="s">
+        <v>2043</v>
+      </c>
+    </row>
+    <row r="631" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A631" s="1" t="s">
+        <v>2044</v>
+      </c>
+      <c r="B631" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C631" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D631" s="0" t="s">
+        <v>2045</v>
+      </c>
+      <c r="E631" s="0" t="s">
+        <v>2046</v>
+      </c>
+    </row>
+    <row r="632" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A632" s="1" t="s">
+        <v>2047</v>
+      </c>
+      <c r="B632" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C632" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D632" s="0" t="s">
+        <v>2048</v>
+      </c>
+      <c r="E632" s="0" t="s">
+        <v>2049</v>
+      </c>
+    </row>
+    <row r="633" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A633" s="1" t="s">
+        <v>2050</v>
+      </c>
+      <c r="B633" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C633" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D633" s="0" t="s">
+        <v>2051</v>
+      </c>
+      <c r="E633" s="0" t="s">
+        <v>2052</v>
+      </c>
+    </row>
+    <row r="634" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A634" s="1" t="s">
+        <v>2053</v>
+      </c>
+      <c r="B634" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C634" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D634" s="0" t="s">
+        <v>2054</v>
+      </c>
+      <c r="E634" s="0" t="s">
+        <v>2055</v>
+      </c>
+    </row>
+    <row r="635" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A635" s="1" t="s">
+        <v>2056</v>
+      </c>
+      <c r="B635" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C635" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D635" s="0" t="s">
+        <v>2057</v>
+      </c>
+      <c r="E635" s="0" t="s">
+        <v>2058</v>
+      </c>
+    </row>
+    <row r="636" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A636" s="1" t="s">
+        <v>2059</v>
+      </c>
+      <c r="B636" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C636" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D636" s="0" t="s">
+        <v>2060</v>
+      </c>
+      <c r="E636" s="0" t="s">
+        <v>2061</v>
+      </c>
+    </row>
+    <row r="637" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A637" s="1" t="s">
+        <v>2062</v>
+      </c>
+      <c r="B637" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C637" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D637" s="0" t="s">
+        <v>2063</v>
+      </c>
+      <c r="E637" s="0" t="s">
+        <v>2064</v>
+      </c>
+    </row>
+    <row r="638" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A638" s="1" t="s">
+        <v>2065</v>
+      </c>
+      <c r="B638" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C638" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D638" s="0" t="s">
+        <v>2066</v>
+      </c>
+      <c r="E638" s="0" t="s">
+        <v>2067</v>
+      </c>
+    </row>
+    <row r="639" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A639" s="1" t="s">
+        <v>2068</v>
+      </c>
+      <c r="B639" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C639" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D639" s="0" t="s">
+        <v>2069</v>
+      </c>
+      <c r="E639" s="0" t="s">
+        <v>2070</v>
+      </c>
+    </row>
+    <row r="640" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A640" s="1" t="s">
+        <v>2071</v>
+      </c>
+      <c r="B640" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C640" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D640" s="0" t="s">
+        <v>2072</v>
+      </c>
+      <c r="E640" s="0" t="s">
+        <v>2073</v>
+      </c>
+    </row>
+    <row r="641" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A641" s="1" t="s">
+        <v>2074</v>
+      </c>
+      <c r="B641" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C641" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D641" s="0" t="s">
+        <v>2075</v>
+      </c>
+      <c r="E641" s="0" t="s">
+        <v>2076</v>
+      </c>
+    </row>
+    <row r="642" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A642" s="1" t="s">
+        <v>2077</v>
+      </c>
+      <c r="B642" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C642" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D642" s="0" t="s">
+        <v>2078</v>
+      </c>
+      <c r="E642" s="0" t="s">
+        <v>2079</v>
+      </c>
+    </row>
+    <row r="643" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A643" s="1" t="s">
+        <v>2080</v>
+      </c>
+      <c r="B643" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C643" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D643" s="0" t="s">
+        <v>2081</v>
+      </c>
+      <c r="E643" s="0" t="s">
+        <v>2082</v>
+      </c>
+    </row>
+    <row r="644" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A644" s="1" t="s">
+        <v>2083</v>
+      </c>
+      <c r="B644" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C644" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D644" s="0" t="s">
+        <v>2084</v>
+      </c>
+      <c r="E644" s="0" t="s">
+        <v>2085</v>
+      </c>
+    </row>
+    <row r="645" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A645" s="1" t="s">
+        <v>2086</v>
+      </c>
+      <c r="B645" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C645" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D645" s="0" t="s">
+        <v>2087</v>
+      </c>
+      <c r="E645" s="0" t="s">
+        <v>2088</v>
+      </c>
+    </row>
+    <row r="646" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A646" s="1" t="s">
+        <v>2089</v>
+      </c>
+      <c r="B646" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C646" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D646" s="0" t="s">
+        <v>2090</v>
+      </c>
+      <c r="E646" s="0" t="s">
+        <v>2091</v>
+      </c>
+    </row>
+    <row r="647" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A647" s="1" t="s">
+        <v>2092</v>
+      </c>
+      <c r="B647" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C647" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D647" s="0" t="s">
+        <v>2093</v>
+      </c>
+      <c r="E647" s="0" t="s">
+        <v>2094</v>
+      </c>
+    </row>
+    <row r="648" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A648" s="1" t="s">
+        <v>2095</v>
+      </c>
+      <c r="B648" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C648" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D648" s="0" t="s">
+        <v>2096</v>
+      </c>
+      <c r="E648" s="0" t="s">
+        <v>2097</v>
+      </c>
+    </row>
+    <row r="649" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A649" s="1" t="s">
+        <v>2098</v>
+      </c>
+      <c r="B649" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C649" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D649" s="0" t="s">
+        <v>2099</v>
+      </c>
+      <c r="E649" s="0" t="s">
+        <v>2100</v>
+      </c>
+    </row>
+    <row r="650" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A650" s="1" t="s">
+        <v>2101</v>
+      </c>
+      <c r="B650" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C650" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D650" s="0" t="s">
+        <v>2102</v>
+      </c>
+      <c r="E650" s="0" t="s">
+        <v>2103</v>
+      </c>
+    </row>
+    <row r="651" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A651" s="1" t="s">
+        <v>2104</v>
+      </c>
+      <c r="B651" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C651" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D651" s="0" t="s">
+        <v>2105</v>
+      </c>
+      <c r="E651" s="0" t="s">
+        <v>2106</v>
+      </c>
+    </row>
+    <row r="652" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A652" s="1" t="s">
+        <v>2107</v>
+      </c>
+      <c r="B652" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C652" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D652" s="0" t="s">
+        <v>2108</v>
+      </c>
+      <c r="E652" s="0" t="s">
+        <v>2109</v>
+      </c>
+    </row>
+    <row r="653" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A653" s="1" t="s">
+        <v>2110</v>
+      </c>
+      <c r="B653" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C653" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D653" s="0" t="s">
+        <v>2111</v>
+      </c>
+      <c r="E653" s="0" t="s">
+        <v>2112</v>
+      </c>
+    </row>
+    <row r="654" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A654" s="1" t="s">
+        <v>2113</v>
+      </c>
+      <c r="B654" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C654" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D654" s="0" t="s">
+        <v>2114</v>
+      </c>
+      <c r="E654" s="0" t="s">
+        <v>2115</v>
+      </c>
+    </row>
+    <row r="655" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A655" s="1" t="s">
+        <v>2116</v>
+      </c>
+      <c r="B655" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C655" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D655" s="0" t="s">
+        <v>2117</v>
+      </c>
+      <c r="E655" s="0" t="s">
+        <v>2118</v>
+      </c>
+    </row>
+    <row r="656" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A656" s="1" t="s">
+        <v>2119</v>
+      </c>
+      <c r="B656" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C656" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D656" s="0" t="s">
+        <v>2120</v>
+      </c>
+      <c r="E656" s="0" t="s">
+        <v>2121</v>
+      </c>
+    </row>
+    <row r="657" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A657" s="1" t="s">
+        <v>2122</v>
+      </c>
+      <c r="B657" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C657" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D657" s="0" t="s">
+        <v>2123</v>
+      </c>
+      <c r="E657" s="0" t="s">
+        <v>2124</v>
+      </c>
+    </row>
+    <row r="658" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A658" s="1" t="s">
+        <v>2125</v>
+      </c>
+      <c r="B658" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C658" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D658" s="0" t="s">
+        <v>2126</v>
+      </c>
+      <c r="E658" s="0" t="s">
+        <v>2127</v>
+      </c>
+    </row>
+    <row r="659" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A659" s="1" t="s">
+        <v>2128</v>
+      </c>
+      <c r="B659" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C659" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D659" s="0" t="s">
+        <v>2129</v>
+      </c>
+      <c r="E659" s="0" t="s">
+        <v>2130</v>
+      </c>
+    </row>
+    <row r="660" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A660" s="1" t="s">
+        <v>2131</v>
+      </c>
+      <c r="B660" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C660" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D660" s="0" t="s">
+        <v>2132</v>
+      </c>
+      <c r="E660" s="0" t="s">
+        <v>2133</v>
+      </c>
+    </row>
+    <row r="661" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A661" s="1" t="s">
+        <v>2134</v>
+      </c>
+      <c r="B661" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C661" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D661" s="0" t="s">
+        <v>2135</v>
+      </c>
+      <c r="E661" s="0" t="s">
+        <v>2136</v>
+      </c>
+    </row>
+    <row r="662" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A662" s="1" t="s">
+        <v>2137</v>
+      </c>
+      <c r="B662" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C662" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D662" s="0" t="s">
+        <v>2138</v>
+      </c>
+      <c r="E662" s="0" t="s">
+        <v>2139</v>
+      </c>
+    </row>
+    <row r="663" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A663" s="1" t="s">
+        <v>2140</v>
+      </c>
+      <c r="B663" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C663" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D663" s="0" t="s">
+        <v>2141</v>
+      </c>
+      <c r="E663" s="0" t="s">
+        <v>2142</v>
+      </c>
+    </row>
+    <row r="664" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A664" s="1" t="s">
+        <v>2143</v>
+      </c>
+      <c r="B664" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C664" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D664" s="0" t="s">
+        <v>2144</v>
+      </c>
+      <c r="E664" s="0" t="s">
+        <v>2145</v>
+      </c>
+    </row>
+    <row r="665" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A665" s="1" t="s">
+        <v>2146</v>
+      </c>
+      <c r="B665" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C665" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D665" s="0" t="s">
+        <v>2147</v>
+      </c>
+      <c r="E665" s="0" t="s">
+        <v>2100</v>
+      </c>
+    </row>
+    <row r="666" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A666" s="1" t="s">
+        <v>2148</v>
+      </c>
+      <c r="B666" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C666" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D666" s="0" t="s">
+        <v>2149</v>
+      </c>
+      <c r="E666" s="0" t="s">
+        <v>2150</v>
+      </c>
+    </row>
+    <row r="667" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A667" s="1" t="s">
+        <v>2151</v>
+      </c>
+      <c r="B667" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C667" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D667" s="0" t="s">
+        <v>2152</v>
+      </c>
+      <c r="E667" s="0" t="s">
+        <v>2153</v>
+      </c>
+    </row>
+    <row r="668" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A668" s="1" t="s">
+        <v>2154</v>
+      </c>
+      <c r="B668" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C668" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D668" s="0" t="s">
+        <v>2155</v>
+      </c>
+      <c r="E668" s="0" t="s">
+        <v>754</v>
+      </c>
+    </row>
+    <row r="669" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A669" s="1" t="s">
+        <v>2156</v>
+      </c>
+      <c r="B669" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C669" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D669" s="0" t="s">
+        <v>2157</v>
+      </c>
+      <c r="E669" s="0" t="s">
+        <v>2158</v>
+      </c>
+    </row>
+    <row r="670" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A670" s="1" t="s">
+        <v>2159</v>
+      </c>
+      <c r="B670" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C670" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D670" s="0" t="s">
+        <v>2160</v>
+      </c>
+      <c r="E670" s="0" t="s">
+        <v>2161</v>
+      </c>
+    </row>
+    <row r="671" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A671" s="1" t="s">
+        <v>2162</v>
+      </c>
+      <c r="B671" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C671" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D671" s="0" t="s">
+        <v>2163</v>
+      </c>
+      <c r="E671" s="0" t="s">
+        <v>2164</v>
+      </c>
+    </row>
+    <row r="672" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A672" s="1" t="s">
+        <v>2165</v>
+      </c>
+      <c r="B672" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C672" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D672" s="0" t="s">
+        <v>2166</v>
+      </c>
+      <c r="E672" s="0" t="s">
+        <v>2167</v>
+      </c>
+    </row>
+    <row r="673" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A673" s="1" t="s">
+        <v>2168</v>
+      </c>
+      <c r="B673" s="1" t="s">
+        <v>1894</v>
+      </c>
+      <c r="C673" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="D673" s="0" t="s">
+        <v>2169</v>
+      </c>
+      <c r="E673" s="0" t="s">
+        <v>2170</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>